<commit_message>
updated llmagent for classifying views
</commit_message>
<xml_diff>
--- a/filtered_views.xlsx
+++ b/filtered_views.xlsx
@@ -459,22 +459,22 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>REV-AMA-05427</t>
+          <t>REV-GOO-05430</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>Amazon</t>
+          <t>Google Locations</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>Anker 65W GaN Fast Charger</t>
+          <t>Metropolitan Dental Health Clinic</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>Highest recommendation! Customer support was also fantastic when I had a quick question about settings. 10/10 purchase. Thanks to the team for the prompt service!</t>
+          <t>World-class care and professionalism. The staff went above and beyond to make me feel comfortable and at ease. Cannot recommend highly enough! #verifiedpurchase</t>
         </is>
       </c>
       <c r="F2" t="n">
@@ -482,11 +482,11 @@
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>20.03.2023</t>
+          <t>11.09.2022</t>
         </is>
       </c>
       <c r="H2" t="n">
-        <v>45</v>
+        <v>48</v>
       </c>
     </row>
     <row r="3">
@@ -495,22 +495,22 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>REV-AMA-00288</t>
+          <t>REV-GOO-03395</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Amazon</t>
+          <t>Google Locations</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>Anker 65W GaN Fast Charger</t>
+          <t>Metropolitan Dental Health Clinic</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>Remarkable craftsmanship. Every detail feels thoughtful and refined. I use it every single day and couldn't be happier with it. #verifiedpurchase</t>
+          <t>Bought this recently. Outstanding service and honest pricing. They diagnosed my car issue accurately, fixed it within hours, and charged less than estimated. Found my forever mechanic!</t>
         </is>
       </c>
       <c r="F3" t="n">
@@ -518,11 +518,11 @@
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>15.08.2023</t>
+          <t>06.03.2024</t>
         </is>
       </c>
       <c r="H3" t="n">
-        <v>43</v>
+        <v>45</v>
       </c>
     </row>
     <row r="4">
@@ -531,22 +531,22 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>REV-AMA-03823</t>
+          <t>REV-GOO-00189</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Amazon</t>
+          <t>Google Locations</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>Anker 65W GaN Fast Charger</t>
+          <t>Metropolitan Dental Health Clinic</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>Review update after 3 months: Five stars without hesitation! Incredible value, intuitive controls, and crystal-clear performance. You cannot beat this at this price point.</t>
+          <t>Incredible place to visit! Breathtaking flora, immaculately manicured gardens, and peaceful tranquility. Truly an oasis in the city. Hope this review helps someone make up their mind.</t>
         </is>
       </c>
       <c r="F4" t="n">
@@ -554,7 +554,7 @@
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>10.07.2022</t>
+          <t>22.12.2023</t>
         </is>
       </c>
       <c r="H4" t="n">
@@ -567,22 +567,22 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>REV-AMA-04210</t>
+          <t>REV-GOO-00714</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>Amazon</t>
+          <t>Google Locations</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>Anker 65W GaN Fast Charger</t>
+          <t>Metropolitan Dental Health Clinic</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>Honestly, game changer! saves me so much time and effort. i have already recommended it to several colleagues and family members.</t>
+          <t>World-class care and professionalism. The staff went above and beyond to make me feel comfortable and at ease. Cannot recommend highly enough! Would definitely recommend checking it out!</t>
         </is>
       </c>
       <c r="F5" t="n">
@@ -590,11 +590,11 @@
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>11.05.2023</t>
+          <t>20.09.2022</t>
         </is>
       </c>
       <c r="H5" t="n">
-        <v>43</v>
+        <v>38</v>
       </c>
     </row>
     <row r="6">
@@ -603,22 +603,22 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>REV-AMA-02251</t>
+          <t>REV-GOO-01771</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>Amazon</t>
+          <t>Google Locations</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>Anker 65W GaN Fast Charger</t>
+          <t>Metropolitan Dental Health Clinic</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>Absolute perfection! Easily the best purchase I have made this year. High quality materials, elegant design, and works flawlessly. Packaging was decent.</t>
+          <t>Review update after 3 months: Best coffee in town by a mile! The baristas are true craftsmen, beans are freshly roasted, and the avocado toast was divine. A 10/10 hidden gem.</t>
         </is>
       </c>
       <c r="F6" t="n">
@@ -626,11 +626,11 @@
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>12.02.2024</t>
+          <t>30.08.2022</t>
         </is>
       </c>
       <c r="H6" t="n">
-        <v>41</v>
+        <v>37</v>
       </c>
     </row>
     <row r="7">
@@ -639,22 +639,22 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>REV-AMA-00163</t>
+          <t>REV-GOO-02055</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>Amazon</t>
+          <t>Google Locations</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>Anker 65W GaN Fast Charger</t>
+          <t>Metropolitan Dental Health Clinic</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>Game changer! Saves me so much time and effort. I have already recommended it to several colleagues and family members. #verifiedpurchase</t>
+          <t>Exceptional service from check-in to departure. The staff treated us like royalty, the suite was gorgeous with breathtaking views, and the spa was heavenly. #verifiedpurchase</t>
         </is>
       </c>
       <c r="F7" t="n">
@@ -662,7 +662,7 @@
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>20.01.2024</t>
+          <t>31.07.2022</t>
         </is>
       </c>
       <c r="H7" t="n">
@@ -675,22 +675,22 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>REV-AMA-02924</t>
+          <t>REV-GOO-02647</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>Amazon</t>
+          <t>Google Locations</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>Anker 65W GaN Fast Charger</t>
+          <t>Metropolitan Dental Health Clinic</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>Summary: Remarkable craftsmanship. Every detail feels thoughtful and refined. I use it every single day and couldn't be happier with it.</t>
+          <t>Outstanding service and honest pricing. They diagnosed my car issue accurately, fixed it within hours, and charged less than estimated. Found my forever mechanic! Hope this review helps someone make up their mind.</t>
         </is>
       </c>
       <c r="F8" t="n">
@@ -698,11 +698,11 @@
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>29.11.2023</t>
+          <t>05.04.2023</t>
         </is>
       </c>
       <c r="H8" t="n">
-        <v>33</v>
+        <v>36</v>
       </c>
     </row>
     <row r="9">
@@ -711,22 +711,22 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>REV-AMA-04084</t>
+          <t>REV-GOO-00273</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>Amazon</t>
+          <t>Google Locations</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>Anker 65W GaN Fast Charger</t>
+          <t>Metropolitan Dental Health Clinic</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>Summary: Remarkable craftsmanship. Every detail feels thoughtful and refined. I use it every single day and couldn't be happier with it.</t>
+          <t>Exceptional service from check-in to departure. The staff treated us like royalty, the suite was gorgeous with breathtaking views, and the spa was heavenly. #verifiedpurchase</t>
         </is>
       </c>
       <c r="F9" t="n">
@@ -734,11 +734,11 @@
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>01.01.2025</t>
+          <t>17.07.2023</t>
         </is>
       </c>
       <c r="H9" t="n">
-        <v>33</v>
+        <v>34</v>
       </c>
     </row>
     <row r="10">
@@ -747,22 +747,22 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>REV-AMA-05055</t>
+          <t>REV-GOO-04288</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>Amazon</t>
+          <t>Google Locations</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>Anker 65W GaN Fast Charger</t>
+          <t>Metropolitan Dental Health Clinic</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>Summary: Flawless performance. Quiet, efficient, and beautifully built. Best in class hands down!</t>
+          <t>Outstanding service and honest pricing. They diagnosed my car issue accurately, fixed it within hours, and charged less than estimated. Found my forever mechanic! #verifiedpurchase</t>
         </is>
       </c>
       <c r="F10" t="n">
@@ -770,11 +770,11 @@
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>20.02.2022</t>
+          <t>16.11.2023</t>
         </is>
       </c>
       <c r="H10" t="n">
-        <v>33</v>
+        <v>34</v>
       </c>
     </row>
     <row r="11">
@@ -783,22 +783,22 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>REV-AMA-00190</t>
+          <t>REV-GOO-05581</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>Amazon</t>
+          <t>Google Locations</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>Anker 65W GaN Fast Charger</t>
+          <t>Metropolitan Dental Health Clinic</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>Review update after 3 months: Absolute perfection! Easily the best purchase I have made this year. High quality materials, elegant design, and works flawlessly.</t>
+          <t>Bought this recently. Phenomenal dining experience! Every course was a culinary masterpiece, the service was impeccable, and the ambience was magical. Best restaurant in the city!</t>
         </is>
       </c>
       <c r="F11" t="n">
@@ -806,11 +806,11 @@
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>23.01.2024</t>
+          <t>28.01.2023</t>
         </is>
       </c>
       <c r="H11" t="n">
-        <v>27</v>
+        <v>32</v>
       </c>
     </row>
     <row r="12">
@@ -819,22 +819,22 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>REV-AMA-03834</t>
+          <t>REV-GOO-00552</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>Amazon</t>
+          <t>Google Locations</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>Anker 65W GaN Fast Charger</t>
+          <t>Metropolitan Dental Health Clinic</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>Outstanding! Exceeded all my expectations. The build quality is top-tier, performance is blazing fast, and battery life is simply phenomenal. Packaging was decent.</t>
+          <t>Honestly, best coffee in town by a mile! the baristas are true craftsmen, beans are freshly roasted, and the avocado toast was divine. a 10/10 hidden gem.</t>
         </is>
       </c>
       <c r="F12" t="n">
@@ -842,11 +842,11 @@
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>10.03.2022</t>
+          <t>13.09.2024</t>
         </is>
       </c>
       <c r="H12" t="n">
-        <v>23</v>
+        <v>31</v>
       </c>
     </row>
     <row r="13">
@@ -855,22 +855,22 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>REV-AMA-01608</t>
+          <t>REV-GOO-06140</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>Amazon</t>
+          <t>Google Locations</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>Anker 65W GaN Fast Charger</t>
+          <t>Metropolitan Dental Health Clinic</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>Honestly, remarkable craftsmanship. every detail feels thoughtful and refined. i use it every single day and couldn't be happier with it.</t>
+          <t>Absolute 5-star experience! Our server was knowledgeable, friendly, and timed each dish to perfection. The flavors were vibrant and authentic. Hope this review helps someone make up their mind.</t>
         </is>
       </c>
       <c r="F13" t="n">
@@ -878,11 +878,11 @@
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>21.03.2023</t>
+          <t>05.01.2022</t>
         </is>
       </c>
       <c r="H13" t="n">
-        <v>22</v>
+        <v>31</v>
       </c>
     </row>
     <row r="14">
@@ -891,22 +891,22 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>REV-AMA-03490</t>
+          <t>REV-GOO-01123</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>Amazon</t>
+          <t>Google Locations</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>Anker 65W GaN Fast Charger</t>
+          <t>Metropolitan Dental Health Clinic</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>Bought this recently. Superb product! Packaging was pristine, delivery was super quick, and it works straight out of the box without any hassle. A+++</t>
+          <t>Honestly, phenomenal dining experience! every course was a culinary masterpiece, the service was impeccable, and the ambience was magical. best restaurant in the city!</t>
         </is>
       </c>
       <c r="F14" t="n">
@@ -914,11 +914,11 @@
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>27.01.2022</t>
+          <t>01.05.2022</t>
         </is>
       </c>
       <c r="H14" t="n">
-        <v>21</v>
+        <v>29</v>
       </c>
     </row>
     <row r="15">
@@ -927,22 +927,22 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>REV-AMA-05187</t>
+          <t>REV-GOO-01192</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>Amazon</t>
+          <t>Google Locations</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>Anker 65W GaN Fast Charger</t>
+          <t>Metropolitan Dental Health Clinic</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>Summary: Absolute perfection! Easily the best purchase I have made this year. High quality materials, elegant design, and works flawlessly.</t>
+          <t>Review update after 3 months: Absolute 5-star experience! Our server was knowledgeable, friendly, and timed each dish to perfection. The flavors were vibrant and authentic.</t>
         </is>
       </c>
       <c r="F15" t="n">
@@ -950,11 +950,11 @@
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>07.09.2024</t>
+          <t>06.12.2023</t>
         </is>
       </c>
       <c r="H15" t="n">
-        <v>19</v>
+        <v>29</v>
       </c>
     </row>
     <row r="16">
@@ -963,22 +963,22 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>REV-AMA-01913</t>
+          <t>REV-GOO-00553</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>Amazon</t>
+          <t>Google Locations</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>Anker 65W GaN Fast Charger</t>
+          <t>Metropolitan Dental Health Clinic</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>Game changer! Saves me so much time and effort. I have already recommended it to several colleagues and family members. Hope this review helps someone make up their mind.</t>
+          <t>Absolute 5-star experience! Our server was knowledgeable, friendly, and timed each dish to perfection. The flavors were vibrant and authentic. Hope this review helps someone make up their mind.</t>
         </is>
       </c>
       <c r="F16" t="n">
@@ -986,11 +986,11 @@
       </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t>16.01.2023</t>
+          <t>21.01.2023</t>
         </is>
       </c>
       <c r="H16" t="n">
-        <v>14</v>
+        <v>27</v>
       </c>
     </row>
     <row r="17">
@@ -999,22 +999,22 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>REV-AMA-05751</t>
+          <t>REV-GOO-01747</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>Amazon</t>
+          <t>Google Locations</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>Anker 65W GaN Fast Charger</t>
+          <t>Metropolitan Dental Health Clinic</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>Flawless performance. Quiet, efficient, and beautifully built. Best in class hands down! Packaging was decent.</t>
+          <t>Summary: Best coffee in town by a mile! The baristas are true craftsmen, beans are freshly roasted, and the avocado toast was divine. A 10/10 hidden gem.</t>
         </is>
       </c>
       <c r="F17" t="n">
@@ -1022,11 +1022,11 @@
       </c>
       <c r="G17" t="inlineStr">
         <is>
-          <t>26.04.2024</t>
+          <t>19.03.2024</t>
         </is>
       </c>
       <c r="H17" t="n">
-        <v>14</v>
+        <v>27</v>
       </c>
     </row>
     <row r="18">
@@ -1035,22 +1035,22 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>REV-AMA-01414</t>
+          <t>REV-GOO-05630</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>Amazon</t>
+          <t>Google Locations</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>Anker 65W GaN Fast Charger</t>
+          <t>Metropolitan Dental Health Clinic</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>Highest recommendation! Customer support was also fantastic when I had a quick question about settings. 10/10 purchase. Packaging was decent.</t>
+          <t>Phenomenal dining experience! Every course was a culinary masterpiece, the service was impeccable, and the ambience was magical. Best restaurant in the city! Thanks to the team for the prompt service!</t>
         </is>
       </c>
       <c r="F18" t="n">
@@ -1058,11 +1058,11 @@
       </c>
       <c r="G18" t="inlineStr">
         <is>
-          <t>19.07.2022</t>
+          <t>20.11.2023</t>
         </is>
       </c>
       <c r="H18" t="n">
-        <v>13</v>
+        <v>27</v>
       </c>
     </row>
     <row r="19">
@@ -1071,22 +1071,22 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>REV-AMA-02790</t>
+          <t>REV-GOO-05968</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>Amazon</t>
+          <t>Google Locations</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>Anker 65W GaN Fast Charger</t>
+          <t>Metropolitan Dental Health Clinic</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>Superb product! Packaging was pristine, delivery was super quick, and it works straight out of the box without any hassle. A+++ Hope this review helps someone make up their mind.</t>
+          <t>Bought this recently. World-class care and professionalism. The staff went above and beyond to make me feel comfortable and at ease. Cannot recommend highly enough!</t>
         </is>
       </c>
       <c r="F19" t="n">
@@ -1094,11 +1094,11 @@
       </c>
       <c r="G19" t="inlineStr">
         <is>
-          <t>27.02.2022</t>
+          <t>04.11.2024</t>
         </is>
       </c>
       <c r="H19" t="n">
-        <v>13</v>
+        <v>25</v>
       </c>
     </row>
     <row r="20">
@@ -1107,22 +1107,22 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>REV-AMA-05831</t>
+          <t>REV-GOO-01159</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>Amazon</t>
+          <t>Google Locations</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>Anker 65W GaN Fast Charger</t>
+          <t>Metropolitan Dental Health Clinic</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>Highest recommendation! Customer support was also fantastic when I had a quick question about settings. 10/10 purchase. Packaging was decent.</t>
+          <t>Bought this recently. Phenomenal dining experience! Every course was a culinary masterpiece, the service was impeccable, and the ambience was magical. Best restaurant in the city!</t>
         </is>
       </c>
       <c r="F20" t="n">
@@ -1130,11 +1130,11 @@
       </c>
       <c r="G20" t="inlineStr">
         <is>
-          <t>17.05.2024</t>
+          <t>04.10.2022</t>
         </is>
       </c>
       <c r="H20" t="n">
-        <v>13</v>
+        <v>22</v>
       </c>
     </row>
     <row r="21">
@@ -1143,22 +1143,22 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>REV-AMA-01012</t>
+          <t>REV-GOO-05164</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>Amazon</t>
+          <t>Google Locations</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>Anker 65W GaN Fast Charger</t>
+          <t>Metropolitan Dental Health Clinic</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>Highest recommendation! Customer support was also fantastic when I had a quick question about settings. 10/10 purchase. Would definitely recommend checking it out!</t>
+          <t>Bought this recently. Absolute 5-star experience! Our server was knowledgeable, friendly, and timed each dish to perfection. The flavors were vibrant and authentic.</t>
         </is>
       </c>
       <c r="F21" t="n">
@@ -1166,11 +1166,11 @@
       </c>
       <c r="G21" t="inlineStr">
         <is>
-          <t>24.07.2023</t>
+          <t>12.05.2023</t>
         </is>
       </c>
       <c r="H21" t="n">
-        <v>10</v>
+        <v>18</v>
       </c>
     </row>
     <row r="22">
@@ -1179,22 +1179,22 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>REV-AMA-03411</t>
+          <t>REV-GOO-03923</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>Amazon</t>
+          <t>Google Locations</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>Anker 65W GaN Fast Charger</t>
+          <t>Metropolitan Dental Health Clinic</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>Terrible quality! It stopped working completely after just two days of light use. Customer support was unhelpful and refused a refund. Total waste of money. #verifiedpurchase</t>
+          <t>Rude management and hostile attitude towards customers. They charged us hidden fees on our bill that were never disclosed upfront. Would definitely recommend checking it out!</t>
         </is>
       </c>
       <c r="F22" t="n">
@@ -1202,11 +1202,11 @@
       </c>
       <c r="G22" t="inlineStr">
         <is>
-          <t>07.08.2024</t>
+          <t>10.09.2023</t>
         </is>
       </c>
       <c r="H22" t="n">
-        <v>35</v>
+        <v>34</v>
       </c>
     </row>
     <row r="23">
@@ -1215,22 +1215,22 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>REV-AMA-02565</t>
+          <t>REV-GOO-01803</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>Amazon</t>
+          <t>Google Locations</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>Anker 65W GaN Fast Charger</t>
+          <t>Metropolitan Dental Health Clinic</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>Summary: Complete rip-off. Battery life is barely an hour when it advertised ten hours. Save your hard-earned money and look elsewhere.</t>
+          <t>Dirty facilities, loud noise all night, and indifferent staff who clearly did not care about our comfort. Avoid this place. Would definitely recommend checking it out!</t>
         </is>
       </c>
       <c r="F23" t="n">
@@ -1238,11 +1238,11 @@
       </c>
       <c r="G23" t="inlineStr">
         <is>
-          <t>12.09.2022</t>
+          <t>17.04.2024</t>
         </is>
       </c>
       <c r="H23" t="n">
-        <v>34</v>
+        <v>31</v>
       </c>
     </row>
     <row r="24">
@@ -1251,22 +1251,22 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>REV-AMA-02457</t>
+          <t>REV-GOO-06013</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>Amazon</t>
+          <t>Google Locations</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>Anker 65W GaN Fast Charger</t>
+          <t>Metropolitan Dental Health Clinic</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>Do not buy this! Cheap plastic construction, smells terrible out of the box, and doesn't match the description at all. Extremely disappointed.</t>
+          <t>Summary: Extremely unprofessional. Had an appointment booked two weeks in advance, waited 45 minutes past the scheduled time, and was treated rudely by reception.</t>
         </is>
       </c>
       <c r="F24" t="n">
@@ -1274,11 +1274,11 @@
       </c>
       <c r="G24" t="inlineStr">
         <is>
-          <t>26.04.2024</t>
+          <t>02.08.2023</t>
         </is>
       </c>
       <c r="H24" t="n">
-        <v>24</v>
+        <v>30</v>
       </c>
     </row>
     <row r="25">
@@ -1287,22 +1287,22 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>REV-AMA-03201</t>
+          <t>REV-GOO-04326</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>Amazon</t>
+          <t>Google Locations</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>Anker 65W GaN Fast Charger</t>
+          <t>Metropolitan Dental Health Clinic</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>Broke on the first attempt to use it. Very fragile materials and feels like a knock-off dollar store item. Huge regret. Would definitely recommend checking it out!</t>
+          <t>Total rip-off. Paid premium prices expecting quality service, but received negligent attention and sub-par quality. Stay far away. Would definitely recommend checking it out!</t>
         </is>
       </c>
       <c r="F25" t="n">
@@ -1310,11 +1310,11 @@
       </c>
       <c r="G25" t="inlineStr">
         <is>
-          <t>03.10.2023</t>
+          <t>15.06.2023</t>
         </is>
       </c>
       <c r="H25" t="n">
-        <v>17</v>
+        <v>28</v>
       </c>
     </row>
     <row r="26">
@@ -1323,22 +1323,22 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>REV-AMA-02132</t>
+          <t>REV-GOO-00533</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>Amazon</t>
+          <t>Google Locations</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>Anker 65W GaN Fast Charger</t>
+          <t>Metropolitan Dental Health Clinic</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>Terrible quality! It stopped working completely after just two days of light use. Customer support was unhelpful and refused a refund. Total waste of money. Packaging was decent.</t>
+          <t>Review update after 3 months: Dirty facilities, loud noise all night, and indifferent staff who clearly did not care about our comfort. Avoid this place.</t>
         </is>
       </c>
       <c r="F26" t="n">
@@ -1346,7 +1346,7 @@
       </c>
       <c r="G26" t="inlineStr">
         <is>
-          <t>13.01.2023</t>
+          <t>21.04.2024</t>
         </is>
       </c>
       <c r="H26" t="n">
@@ -1359,22 +1359,22 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>REV-AMA-04991</t>
+          <t>REV-GOO-01334</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>Amazon</t>
+          <t>Google Locations</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>Anker 65W GaN Fast Charger</t>
+          <t>Metropolitan Dental Health Clinic</t>
         </is>
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>Do not buy this! Cheap plastic construction, smells terrible out of the box, and doesn't match the description at all. Extremely disappointed. Thanks to the team for the prompt service!</t>
+          <t>Extremely unprofessional. Had an appointment booked two weeks in advance, waited 45 minutes past the scheduled time, and was treated rudely by reception. Thanks to the team for the prompt service!</t>
         </is>
       </c>
       <c r="F27" t="n">
@@ -1382,11 +1382,11 @@
       </c>
       <c r="G27" t="inlineStr">
         <is>
-          <t>13.11.2023</t>
+          <t>04.01.2024</t>
         </is>
       </c>
       <c r="H27" t="n">
-        <v>9</v>
+        <v>14</v>
       </c>
     </row>
     <row r="28">
@@ -1395,22 +1395,22 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>REV-AMA-01545</t>
+          <t>REV-GOO-00490</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>Amazon</t>
+          <t>Google Locations</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>Anker 65W GaN Fast Charger</t>
+          <t>Metropolitan Dental Health Clinic</t>
         </is>
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>Customer service was a nightmare. Product died in a week, and they kept giving me the runaround instead of honoring the warranty.</t>
+          <t>Bought this recently. Total rip-off. Paid premium prices expecting quality service, but received negligent attention and sub-par quality. Stay far away.</t>
         </is>
       </c>
       <c r="F28" t="n">
@@ -1418,11 +1418,11 @@
       </c>
       <c r="G28" t="inlineStr">
         <is>
-          <t>26.09.2023</t>
+          <t>08.05.2024</t>
         </is>
       </c>
       <c r="H28" t="n">
-        <v>8</v>
+        <v>5</v>
       </c>
     </row>
     <row r="29">
@@ -1431,22 +1431,22 @@
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>REV-AMA-01757</t>
+          <t>REV-GOO-04294</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>Amazon</t>
+          <t>Google Locations</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>Anker 65W GaN Fast Charger</t>
+          <t>Metropolitan Dental Health Clinic</t>
         </is>
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>Summary: Complete rip-off. Battery life is barely an hour when it advertised ten hours. Save your hard-earned money and look elsewhere.</t>
+          <t>Worst dining experience of my life. The server was rude, food took over an hour to arrive, and when it did, the steak was cold and burnt. Packaging was decent.</t>
         </is>
       </c>
       <c r="F29" t="n">
@@ -1454,11 +1454,11 @@
       </c>
       <c r="G29" t="inlineStr">
         <is>
-          <t>31.01.2024</t>
+          <t>03.02.2024</t>
         </is>
       </c>
       <c r="H29" t="n">
-        <v>8</v>
+        <v>5</v>
       </c>
     </row>
     <row r="30">
@@ -1467,22 +1467,22 @@
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>REV-AMA-02416</t>
+          <t>REV-GOO-05854</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>Amazon</t>
+          <t>Google Locations</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>Anker 65W GaN Fast Charger</t>
+          <t>Metropolitan Dental Health Clinic</t>
         </is>
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>Terrible quality! It stopped working completely after just two days of light use. Customer support was unhelpful and refused a refund. Total waste of money. Would definitely recommend checking it out!</t>
+          <t>Total rip-off. Paid premium prices expecting quality service, but received negligent attention and sub-par quality. Stay far away. Hope this review helps someone make up their mind.</t>
         </is>
       </c>
       <c r="F30" t="n">
@@ -1490,11 +1490,11 @@
       </c>
       <c r="G30" t="inlineStr">
         <is>
-          <t>09.07.2024</t>
+          <t>04.05.2023</t>
         </is>
       </c>
       <c r="H30" t="n">
-        <v>8</v>
+        <v>4</v>
       </c>
     </row>
     <row r="31">
@@ -1503,22 +1503,22 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>REV-AMA-05069</t>
+          <t>REV-GOO-00160</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>Amazon</t>
+          <t>Google Locations</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>Anker 65W GaN Fast Charger</t>
+          <t>Metropolitan Dental Health Clinic</t>
         </is>
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>Arrived damaged with a broken seal. Tried to use it anyway, and it immediately overheated. Returning this junk ASAP! Thanks to the team for the prompt service!</t>
+          <t>Rude management and hostile attitude towards customers. They charged us hidden fees on our bill that were never disclosed upfront. Packaging was decent.</t>
         </is>
       </c>
       <c r="F31" t="n">
@@ -1526,11 +1526,11 @@
       </c>
       <c r="G31" t="inlineStr">
         <is>
-          <t>10.02.2023</t>
+          <t>26.12.2022</t>
         </is>
       </c>
       <c r="H31" t="n">
-        <v>6</v>
+        <v>3</v>
       </c>
     </row>
     <row r="32">
@@ -1539,22 +1539,22 @@
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>REV-AMA-02675</t>
+          <t>REV-GOO-00422</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>Amazon</t>
+          <t>Google Locations</t>
         </is>
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>Anker 65W GaN Fast Charger</t>
+          <t>Metropolitan Dental Health Clinic</t>
         </is>
       </c>
       <c r="E32" t="inlineStr">
         <is>
-          <t>Bought this recently. Customer service was a nightmare. Product died in a week, and they kept giving me the runaround instead of honoring the warranty.</t>
+          <t>Honestly, rude management and hostile attitude towards customers. they charged us hidden fees on our bill that were never disclosed upfront.</t>
         </is>
       </c>
       <c r="F32" t="n">
@@ -1562,11 +1562,11 @@
       </c>
       <c r="G32" t="inlineStr">
         <is>
-          <t>15.01.2022</t>
+          <t>18.06.2024</t>
         </is>
       </c>
       <c r="H32" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
     </row>
     <row r="33">
@@ -1575,22 +1575,22 @@
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>REV-AMA-03198</t>
+          <t>REV-GOO-01812</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>Amazon</t>
+          <t>Google Locations</t>
         </is>
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>Anker 65W GaN Fast Charger</t>
+          <t>Metropolitan Dental Health Clinic</t>
         </is>
       </c>
       <c r="E33" t="inlineStr">
         <is>
-          <t>Defective right out of the packaging. The buttons are stiff and don't respond half the time. Regret purchasing this entirely. Hope this review helps someone make up their mind.</t>
+          <t>Overpriced and incredibly underwhelming. The portions were tiny, tasteless, and our orders were mixed up twice. Do not recommend.</t>
         </is>
       </c>
       <c r="F33" t="n">
@@ -1598,11 +1598,11 @@
       </c>
       <c r="G33" t="inlineStr">
         <is>
-          <t>19.06.2024</t>
+          <t>17.04.2023</t>
         </is>
       </c>
       <c r="H33" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
     </row>
     <row r="34">
@@ -1611,22 +1611,22 @@
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>REV-AMA-04911</t>
+          <t>REV-GOO-02784</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>Amazon</t>
+          <t>Google Locations</t>
         </is>
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>Anker 65W GaN Fast Charger</t>
+          <t>Metropolitan Dental Health Clinic</t>
         </is>
       </c>
       <c r="E34" t="inlineStr">
         <is>
-          <t>Arrived damaged with a broken seal. Tried to use it anyway, and it immediately overheated. Returning this junk ASAP!</t>
+          <t>Never coming back here! The staff was dismissive, the room smelled of damp mold, and the AC was broken during a heatwave. Disastrous stay. Would definitely recommend checking it out!</t>
         </is>
       </c>
       <c r="F34" t="n">
@@ -1634,11 +1634,11 @@
       </c>
       <c r="G34" t="inlineStr">
         <is>
-          <t>01.11.2024</t>
+          <t>20.08.2022</t>
         </is>
       </c>
       <c r="H34" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
     </row>
     <row r="35">
@@ -1647,22 +1647,22 @@
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>REV-AMA-04996</t>
+          <t>REV-GOO-04831</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>Amazon</t>
+          <t>Google Locations</t>
         </is>
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>Anker 65W GaN Fast Charger</t>
+          <t>Metropolitan Dental Health Clinic</t>
         </is>
       </c>
       <c r="E35" t="inlineStr">
         <is>
-          <t>Honestly, awful product. failed right after the return window closed. classic planned obsolescence. never buying from this brand again.</t>
+          <t>Overpriced and incredibly underwhelming. The portions were tiny, tasteless, and our orders were mixed up twice. Do not recommend. Packaging was decent.</t>
         </is>
       </c>
       <c r="F35" t="n">
@@ -1670,11 +1670,11 @@
       </c>
       <c r="G35" t="inlineStr">
         <is>
-          <t>02.07.2022</t>
+          <t>08.05.2024</t>
         </is>
       </c>
       <c r="H35" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
     </row>
     <row r="36">
@@ -1683,22 +1683,22 @@
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>REV-AMA-03607</t>
+          <t>REV-GOO-05467</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>Amazon</t>
+          <t>Google Locations</t>
         </is>
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>Anker 65W GaN Fast Charger</t>
+          <t>Metropolitan Dental Health Clinic</t>
         </is>
       </c>
       <c r="E36" t="inlineStr">
         <is>
-          <t>Summary: Poor design, frustrating setup instructions, and constantly disconnects. Avoid at all costs!</t>
+          <t>Summary: Extremely unprofessional. Had an appointment booked two weeks in advance, waited 45 minutes past the scheduled time, and was treated rudely by reception.</t>
         </is>
       </c>
       <c r="F36" t="n">
@@ -1706,11 +1706,11 @@
       </c>
       <c r="G36" t="inlineStr">
         <is>
-          <t>09.10.2023</t>
+          <t>08.07.2023</t>
         </is>
       </c>
       <c r="H36" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
     </row>
     <row r="37">
@@ -1719,22 +1719,22 @@
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>REV-AMA-05182</t>
+          <t>REV-GOO-03964</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>Amazon</t>
+          <t>Google Locations</t>
         </is>
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>Anker 65W GaN Fast Charger</t>
+          <t>Metropolitan Dental Health Clinic</t>
         </is>
       </c>
       <c r="E37" t="inlineStr">
         <is>
-          <t>Awful product. Failed right after the return window closed. Classic planned obsolescence. Never buying from this brand again. #verifiedpurchase</t>
+          <t>Rude management and hostile attitude towards customers. They charged us hidden fees on our bill that were never disclosed upfront. Would definitely recommend checking it out!</t>
         </is>
       </c>
       <c r="F37" t="n">
@@ -1742,11 +1742,11 @@
       </c>
       <c r="G37" t="inlineStr">
         <is>
-          <t>08.01.2024</t>
+          <t>02.08.2022</t>
         </is>
       </c>
       <c r="H37" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
     </row>
     <row r="38">
@@ -1755,22 +1755,22 @@
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>REV-AMA-01318</t>
+          <t>REV-GOO-05818</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>Amazon</t>
+          <t>Google Locations</t>
         </is>
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t>Anker 65W GaN Fast Charger</t>
+          <t>Metropolitan Dental Health Clinic</t>
         </is>
       </c>
       <c r="E38" t="inlineStr">
         <is>
-          <t>Arrived damaged with a broken seal. Tried to use it anyway, and it immediately overheated. Returning this junk ASAP! Would definitely recommend checking it out!</t>
+          <t>Worst dining experience of my life. The server was rude, food took over an hour to arrive, and when it did, the steak was cold and burnt. Thanks to the team for the prompt service!</t>
         </is>
       </c>
       <c r="F38" t="n">
@@ -1778,11 +1778,11 @@
       </c>
       <c r="G38" t="inlineStr">
         <is>
-          <t>27.09.2023</t>
+          <t>21.02.2022</t>
         </is>
       </c>
       <c r="H38" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
     </row>
     <row r="39">
@@ -1791,22 +1791,22 @@
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>REV-AMA-05214</t>
+          <t>REV-GOO-00001</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>Amazon</t>
+          <t>Google Locations</t>
         </is>
       </c>
       <c r="D39" t="inlineStr">
         <is>
-          <t>Anker 65W GaN Fast Charger</t>
+          <t>Metropolitan Dental Health Clinic</t>
         </is>
       </c>
       <c r="E39" t="inlineStr">
         <is>
-          <t>Summary: Poor design, frustrating setup instructions, and constantly disconnects. Avoid at all costs!</t>
+          <t>Terrible hygiene and filthy tables. Saw flies around the counter and the bathroom had no soap or paper towels. Health department needs to inspect this. Would definitely recommend checking it out!</t>
         </is>
       </c>
       <c r="F39" t="n">
@@ -1814,11 +1814,11 @@
       </c>
       <c r="G39" t="inlineStr">
         <is>
-          <t>09.02.2023</t>
+          <t>13.10.2022</t>
         </is>
       </c>
       <c r="H39" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="40">
@@ -1827,22 +1827,22 @@
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>REV-AMA-01517</t>
+          <t>REV-GOO-00633</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>Amazon</t>
+          <t>Google Locations</t>
         </is>
       </c>
       <c r="D40" t="inlineStr">
         <is>
-          <t>Anker 65W GaN Fast Charger</t>
+          <t>Metropolitan Dental Health Clinic</t>
         </is>
       </c>
       <c r="E40" t="inlineStr">
         <is>
-          <t>Terrible quality! It stopped working completely after just two days of light use. Customer support was unhelpful and refused a refund. Total waste of money. Would definitely recommend checking it out!</t>
+          <t>Dirty facilities, loud noise all night, and indifferent staff who clearly did not care about our comfort. Avoid this place. Hope this review helps someone make up their mind.</t>
         </is>
       </c>
       <c r="F40" t="n">
@@ -1850,11 +1850,11 @@
       </c>
       <c r="G40" t="inlineStr">
         <is>
-          <t>24.05.2024</t>
+          <t>20.02.2022</t>
         </is>
       </c>
       <c r="H40" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="41">
@@ -1863,22 +1863,22 @@
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>REV-AMA-05783</t>
+          <t>REV-GOO-01041</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>Amazon</t>
+          <t>Google Locations</t>
         </is>
       </c>
       <c r="D41" t="inlineStr">
         <is>
-          <t>Anker 65W GaN Fast Charger</t>
+          <t>Metropolitan Dental Health Clinic</t>
         </is>
       </c>
       <c r="E41" t="inlineStr">
         <is>
-          <t>Do not buy this! Cheap plastic construction, smells terrible out of the box, and doesn't match the description at all. Extremely disappointed. Thanks to the team for the prompt service!</t>
+          <t>Honestly, worst dining experience of my life. the server was rude, food took over an hour to arrive, and when it did, the steak was cold and burnt.</t>
         </is>
       </c>
       <c r="F41" t="n">
@@ -1886,11 +1886,11 @@
       </c>
       <c r="G41" t="inlineStr">
         <is>
-          <t>22.09.2024</t>
+          <t>11.09.2022</t>
         </is>
       </c>
       <c r="H41" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="42">
@@ -1899,22 +1899,22 @@
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>REV-AMA-04957</t>
+          <t>REV-GOO-02746</t>
         </is>
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>Amazon</t>
+          <t>Google Locations</t>
         </is>
       </c>
       <c r="D42" t="inlineStr">
         <is>
-          <t>Anker 65W GaN Fast Charger</t>
+          <t>Metropolitan Dental Health Clinic</t>
         </is>
       </c>
       <c r="E42" t="inlineStr">
         <is>
-          <t>Bought this recently. Expected much better from this brand. Battery drains fast and audio is tinny with zero bass. Two stars because shipping was fast.</t>
+          <t>Disappointing visit. The ambiance is charming, but the food was bland and lukewarm. Service was sluggish throughout the evening.</t>
         </is>
       </c>
       <c r="F42" t="n">
@@ -1922,11 +1922,11 @@
       </c>
       <c r="G42" t="inlineStr">
         <is>
-          <t>26.08.2022</t>
+          <t>22.06.2023</t>
         </is>
       </c>
       <c r="H42" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
     </row>
     <row r="43">
@@ -1935,22 +1935,22 @@
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>REV-AMA-03666</t>
+          <t>REV-GOO-01225</t>
         </is>
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>Amazon</t>
+          <t>Google Locations</t>
         </is>
       </c>
       <c r="D43" t="inlineStr">
         <is>
-          <t>Anker 65W GaN Fast Charger</t>
+          <t>Metropolitan Dental Health Clinic</t>
         </is>
       </c>
       <c r="E43" t="inlineStr">
         <is>
-          <t>Summary: Decent overall, but has noticeable trade-offs. The cord is too short and the instruction booklet is minimal.</t>
+          <t>Honestly, decent spot, nothing extraordinary. the food was okay, service was acceptable, and the prices were fair for the neighborhood.</t>
         </is>
       </c>
       <c r="F43" t="n">
@@ -1958,7 +1958,7 @@
       </c>
       <c r="G43" t="inlineStr">
         <is>
-          <t>31.10.2023</t>
+          <t>23.07.2022</t>
         </is>
       </c>
       <c r="H43" t="n">
@@ -1971,22 +1971,22 @@
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>REV-AMA-04055</t>
+          <t>REV-GOO-03514</t>
         </is>
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>Amazon</t>
+          <t>Google Locations</t>
         </is>
       </c>
       <c r="D44" t="inlineStr">
         <is>
-          <t>Anker 65W GaN Fast Charger</t>
+          <t>Metropolitan Dental Health Clinic</t>
         </is>
       </c>
       <c r="E44" t="inlineStr">
         <is>
-          <t>Underwhelming performance. The main features are buggy and sluggish. It gets lukewarm rather than hot. Not worth the full retail price. Thanks to the team for the prompt service!</t>
+          <t>Average food with very slow service. We waited almost an hour for appetizers. The staff tried hard, but they were clearly understaffed. Packaging was decent.</t>
         </is>
       </c>
       <c r="F44" t="n">
@@ -1994,11 +1994,11 @@
       </c>
       <c r="G44" t="inlineStr">
         <is>
-          <t>12.10.2022</t>
+          <t>18.11.2023</t>
         </is>
       </c>
       <c r="H44" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
     </row>
     <row r="45">
@@ -2007,22 +2007,22 @@
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>REV-AMA-04178</t>
+          <t>REV-GOO-04520</t>
         </is>
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>Amazon</t>
+          <t>Google Locations</t>
         </is>
       </c>
       <c r="D45" t="inlineStr">
         <is>
-          <t>Anker 65W GaN Fast Charger</t>
+          <t>Metropolitan Dental Health Clinic</t>
         </is>
       </c>
       <c r="E45" t="inlineStr">
         <is>
-          <t>Much better than my previous one. Sleek, fast, and intuitive. Dropped one star because the companion app occasionally desyncs. Thanks to the team for the prompt service!</t>
+          <t>Review update after 3 months: Wonderful experience overall. The staff was courteous and accommodating. The rooms were spotless and nicely appointed. Will visit again.</t>
         </is>
       </c>
       <c r="F45" t="n">
@@ -2030,11 +2030,11 @@
       </c>
       <c r="G45" t="inlineStr">
         <is>
-          <t>27.08.2022</t>
+          <t>14.11.2023</t>
         </is>
       </c>
       <c r="H45" t="n">
-        <v>4</v>
+        <v>0</v>
       </c>
     </row>
     <row r="46">
@@ -2043,22 +2043,22 @@
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>REV-AMA-02981</t>
+          <t>REV-GOO-00014</t>
         </is>
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>Amazon</t>
+          <t>Google Locations</t>
         </is>
       </c>
       <c r="D46" t="inlineStr">
         <is>
-          <t>Anker 65W GaN Fast Charger</t>
+          <t>Metropolitan Dental Health Clinic</t>
         </is>
       </c>
       <c r="E46" t="inlineStr">
         <is>
-          <t>Solid 4 stars. Great features and sleek design. The only reason I didn't give 5 stars is because the charging cable is a bit short. Hope this review helps someone make up their mind.</t>
+          <t>Wonderful experience overall. The staff was courteous and accommodating. The rooms were spotless and nicely appointed. Will visit again. Would definitely recommend checking it out!</t>
         </is>
       </c>
       <c r="F46" t="n">
@@ -2066,11 +2066,11 @@
       </c>
       <c r="G46" t="inlineStr">
         <is>
-          <t>01.08.2024</t>
+          <t>23.06.2023</t>
         </is>
       </c>
       <c r="H46" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="47">
@@ -2079,22 +2079,22 @@
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>REV-AMA-02683</t>
+          <t>REV-GOO-01473</t>
         </is>
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>Amazon</t>
+          <t>Google Locations</t>
         </is>
       </c>
       <c r="D47" t="inlineStr">
         <is>
-          <t>Anker 65W GaN Fast Charger</t>
+          <t>Metropolitan Dental Health Clinic</t>
         </is>
       </c>
       <c r="E47" t="inlineStr">
         <is>
-          <t>Impressive performance for the price. Clear sound, crisp buttons, and durable finish. Highly recommended for most people. Thanks to the team for the prompt service!</t>
+          <t>Very enjoyable visit. Loved the artisan coffee and freshly baked pastries. A wonderful quiet corner to read or get work done. Thanks to the team for the prompt service!</t>
         </is>
       </c>
       <c r="F47" t="n">
@@ -2102,11 +2102,11 @@
       </c>
       <c r="G47" t="inlineStr">
         <is>
-          <t>21.03.2023</t>
+          <t>19.06.2022</t>
         </is>
       </c>
       <c r="H47" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
     </row>
     <row r="48">
@@ -2115,22 +2115,22 @@
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>REV-AMA-01288</t>
+          <t>REV-GOO-02730</t>
         </is>
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>Amazon</t>
+          <t>Google Locations</t>
         </is>
       </c>
       <c r="D48" t="inlineStr">
         <is>
-          <t>Anker 65W GaN Fast Charger</t>
+          <t>Metropolitan Dental Health Clinic</t>
         </is>
       </c>
       <c r="E48" t="inlineStr">
         <is>
-          <t>Mediocre at best. It functions, but feels much cheaper than the pictures suggest. Probably won't last more than a few months. Hope this review helps someone make up their mind.</t>
+          <t>Underwhelming experience. The place looks great on social media, but reality falls short. Portions are small and flavors are muted. Packaging was decent.</t>
         </is>
       </c>
       <c r="F48" t="n">
@@ -2138,7 +2138,7 @@
       </c>
       <c r="G48" t="inlineStr">
         <is>
-          <t>16.09.2022</t>
+          <t>06.01.2022</t>
         </is>
       </c>
       <c r="H48" t="n">
@@ -2151,30 +2151,30 @@
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>REV-AMA-02962</t>
+          <t>REV-GOO-04339</t>
         </is>
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>Amazon</t>
+          <t>Google Locations</t>
         </is>
       </c>
       <c r="D49" t="inlineStr">
         <is>
-          <t>Anker 65W GaN Fast Charger</t>
+          <t>Metropolitan Dental Health Clinic</t>
         </is>
       </c>
       <c r="E49" t="inlineStr">
         <is>
-          <t>Average product. It gets the job done for everyday basic use, but nothing to write home about. Decent value for the budget price.</t>
+          <t>Honestly, not worth the hype or the high prices. decent location, but the amenities are outdated and the rooms need urgent renovation.</t>
         </is>
       </c>
       <c r="F49" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="G49" t="inlineStr">
         <is>
-          <t>07.12.2023</t>
+          <t>08.04.2024</t>
         </is>
       </c>
       <c r="H49" t="n">
@@ -2187,22 +2187,22 @@
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>REV-AMA-00424</t>
+          <t>REV-GOO-00856</t>
         </is>
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>Amazon</t>
+          <t>Google Locations</t>
         </is>
       </c>
       <c r="D50" t="inlineStr">
         <is>
-          <t>Anker 65W GaN Fast Charger</t>
+          <t>Metropolitan Dental Health Clinic</t>
         </is>
       </c>
       <c r="E50" t="inlineStr">
         <is>
-          <t>Summary: Average product. It gets the job done for everyday basic use, but nothing to write home about. Decent value for the budget price.</t>
+          <t>Average experience overall. Convenient location and clean space, but parking was a nightmare and wait times were a bit long.</t>
         </is>
       </c>
       <c r="F50" t="n">
@@ -2210,11 +2210,11 @@
       </c>
       <c r="G50" t="inlineStr">
         <is>
-          <t>20.12.2023</t>
+          <t>31.08.2022</t>
         </is>
       </c>
       <c r="H50" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="51">
@@ -2223,34 +2223,34 @@
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>REV-AMA-00069</t>
+          <t>REV-GOO-03015</t>
         </is>
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>Amazon</t>
+          <t>Google Locations</t>
         </is>
       </c>
       <c r="D51" t="inlineStr">
         <is>
-          <t>Anker 65W GaN Fast Charger</t>
+          <t>Metropolitan Dental Health Clinic</t>
         </is>
       </c>
       <c r="E51" t="inlineStr">
         <is>
-          <t>Bought this recently. Much better than my previous one. Sleek, fast, and intuitive. Dropped one star because the companion app occasionally desyncs.</t>
+          <t>Average food with very slow service. We waited almost an hour for appetizers. The staff tried hard, but they were clearly understaffed. Thanks to the team for the prompt service!</t>
         </is>
       </c>
       <c r="F51" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="G51" t="inlineStr">
         <is>
-          <t>23.06.2022</t>
+          <t>31.03.2023</t>
         </is>
       </c>
       <c r="H51" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
     </row>
     <row r="52">
@@ -2259,34 +2259,34 @@
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>REV-AMA-01055</t>
+          <t>REV-GOO-05612</t>
         </is>
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>Amazon</t>
+          <t>Google Locations</t>
         </is>
       </c>
       <c r="D52" t="inlineStr">
         <is>
-          <t>Anker 65W GaN Fast Charger</t>
+          <t>Metropolitan Dental Health Clinic</t>
         </is>
       </c>
       <c r="E52" t="inlineStr">
         <is>
-          <t>Honestly, decent idea, flawed execution. the manual is poorly translated and several promised features are absent or locked behind a paywall.</t>
+          <t>Average experience overall. Convenient location and clean space, but parking was a nightmare and wait times were a bit long. Would definitely recommend checking it out!</t>
         </is>
       </c>
       <c r="F52" t="n">
+        <v>3</v>
+      </c>
+      <c r="G52" t="inlineStr">
+        <is>
+          <t>24.07.2024</t>
+        </is>
+      </c>
+      <c r="H52" t="n">
         <v>2</v>
-      </c>
-      <c r="G52" t="inlineStr">
-        <is>
-          <t>22.04.2023</t>
-        </is>
-      </c>
-      <c r="H52" t="n">
-        <v>15</v>
       </c>
     </row>
     <row r="53">
@@ -2295,34 +2295,34 @@
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>REV-AMA-01937</t>
+          <t>REV-GOO-02241</t>
         </is>
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t>Amazon</t>
+          <t>Google Locations</t>
         </is>
       </c>
       <c r="D53" t="inlineStr">
         <is>
-          <t>Anker 65W GaN Fast Charger</t>
+          <t>Metropolitan Dental Health Clinic</t>
         </is>
       </c>
       <c r="E53" t="inlineStr">
         <is>
-          <t>Much better than my previous one. Sleek, fast, and intuitive. Dropped one star because the companion app occasionally desyncs. Would definitely recommend checking it out!</t>
+          <t>Average experience overall. Convenient location and clean space, but parking was a nightmare and wait times were a bit long. #verifiedpurchase</t>
         </is>
       </c>
       <c r="F53" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="G53" t="inlineStr">
         <is>
-          <t>29.12.2022</t>
+          <t>18.02.2022</t>
         </is>
       </c>
       <c r="H53" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
     </row>
     <row r="54">
@@ -2331,34 +2331,34 @@
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>REV-AMA-05885</t>
+          <t>REV-GOO-05936</t>
         </is>
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t>Amazon</t>
+          <t>Google Locations</t>
         </is>
       </c>
       <c r="D54" t="inlineStr">
         <is>
-          <t>Anker 65W GaN Fast Charger</t>
+          <t>Metropolitan Dental Health Clinic</t>
         </is>
       </c>
       <c r="E54" t="inlineStr">
         <is>
-          <t>Acceptable quality. Does what it says on the box, though battery life is slightly below my expectations. Thanks to the team for the prompt service!</t>
+          <t>Bought this recently. Great meal with friends. Flavorful dishes, generous portions, and vibrant vibe. Only knock was the slightly elevated noise level.</t>
         </is>
       </c>
       <c r="F54" t="n">
+        <v>4</v>
+      </c>
+      <c r="G54" t="inlineStr">
+        <is>
+          <t>26.10.2024</t>
+        </is>
+      </c>
+      <c r="H54" t="n">
         <v>3</v>
-      </c>
-      <c r="G54" t="inlineStr">
-        <is>
-          <t>09.11.2023</t>
-        </is>
-      </c>
-      <c r="H54" t="n">
-        <v>1</v>
       </c>
     </row>
     <row r="55">
@@ -2367,34 +2367,34 @@
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>REV-AMA-02207</t>
+          <t>REV-GOO-03985</t>
         </is>
       </c>
       <c r="C55" t="inlineStr">
         <is>
-          <t>Amazon</t>
+          <t>Google Locations</t>
         </is>
       </c>
       <c r="D55" t="inlineStr">
         <is>
-          <t>Anker 65W GaN Fast Charger</t>
+          <t>Metropolitan Dental Health Clinic</t>
         </is>
       </c>
       <c r="E55" t="inlineStr">
         <is>
-          <t>Very pleased. The build feels premium and it does exactly what I needed it to do. Would happily purchase again. Thanks to the team for the prompt service!</t>
+          <t>Mediocre stay. Cleanliness was questionable and the bed was uncomfortable. Would look for alternative options next time in town. Hope this review helps someone make up their mind.</t>
         </is>
       </c>
       <c r="F55" t="n">
+        <v>2</v>
+      </c>
+      <c r="G55" t="inlineStr">
+        <is>
+          <t>23.01.2024</t>
+        </is>
+      </c>
+      <c r="H55" t="n">
         <v>4</v>
-      </c>
-      <c r="G55" t="inlineStr">
-        <is>
-          <t>29.07.2023</t>
-        </is>
-      </c>
-      <c r="H55" t="n">
-        <v>0</v>
       </c>
     </row>
     <row r="56">
@@ -2403,34 +2403,34 @@
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>REV-AMA-04597</t>
+          <t>REV-GOO-00987</t>
         </is>
       </c>
       <c r="C56" t="inlineStr">
         <is>
-          <t>Amazon</t>
+          <t>Google Locations</t>
         </is>
       </c>
       <c r="D56" t="inlineStr">
         <is>
-          <t>Anker 65W GaN Fast Charger</t>
+          <t>Metropolitan Dental Health Clinic</t>
         </is>
       </c>
       <c r="E56" t="inlineStr">
         <is>
-          <t>Average product. It gets the job done for everyday basic use, but nothing to write home about. Decent value for the budget price. Packaging was decent.</t>
+          <t>High quality service and clean facilities. Doctor and nurses were thorough, gentle, and answered all my questions patiently. Hope this review helps someone make up their mind.</t>
         </is>
       </c>
       <c r="F56" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="G56" t="inlineStr">
         <is>
-          <t>04.09.2022</t>
+          <t>01.03.2023</t>
         </is>
       </c>
       <c r="H56" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
     </row>
     <row r="57">
@@ -2439,22 +2439,22 @@
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>REV-AMA-00236</t>
+          <t>REV-GOO-00109</t>
         </is>
       </c>
       <c r="C57" t="inlineStr">
         <is>
-          <t>Amazon</t>
+          <t>Google Locations</t>
         </is>
       </c>
       <c r="D57" t="inlineStr">
         <is>
-          <t>Anker 65W GaN Fast Charger</t>
+          <t>Metropolitan Dental Health Clinic</t>
         </is>
       </c>
       <c r="E57" t="inlineStr">
         <is>
-          <t>Honestly, great value for money. minor learning curve with the controls, but once configured, it has been reliable every day.</t>
+          <t>Great atmosphere and delicious food! The pasta was freshly handmade and the wine selection was impressive. Service was attentive and friendly. Would definitely recommend checking it out!</t>
         </is>
       </c>
       <c r="F57" t="n">
@@ -2462,11 +2462,11 @@
       </c>
       <c r="G57" t="inlineStr">
         <is>
-          <t>07.02.2024</t>
+          <t>30.08.2023</t>
         </is>
       </c>
       <c r="H57" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
     </row>
     <row r="58">
@@ -2475,34 +2475,34 @@
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>REV-AMA-05482</t>
+          <t>REV-GOO-01139</t>
         </is>
       </c>
       <c r="C58" t="inlineStr">
         <is>
-          <t>Amazon</t>
+          <t>Google Locations</t>
         </is>
       </c>
       <c r="D58" t="inlineStr">
         <is>
-          <t>Anker 65W GaN Fast Charger</t>
+          <t>Metropolitan Dental Health Clinic</t>
         </is>
       </c>
       <c r="E58" t="inlineStr">
         <is>
-          <t>Bought this recently. Expected much better from this brand. Battery drains fast and audio is tinny with zero bass. Two stars because shipping was fast.</t>
+          <t>Beautiful spot for an evening stroll. Well-maintained pathways, lovely landscaping, and safe environment for families. Parking fills up quickly though.</t>
         </is>
       </c>
       <c r="F58" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="G58" t="inlineStr">
         <is>
-          <t>11.05.2023</t>
+          <t>06.11.2023</t>
         </is>
       </c>
       <c r="H58" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="59">
@@ -2511,22 +2511,22 @@
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>REV-AMA-04631</t>
+          <t>REV-GOO-01668</t>
         </is>
       </c>
       <c r="C59" t="inlineStr">
         <is>
-          <t>Amazon</t>
+          <t>Google Locations</t>
         </is>
       </c>
       <c r="D59" t="inlineStr">
         <is>
-          <t>Anker 65W GaN Fast Charger</t>
+          <t>Metropolitan Dental Health Clinic</t>
         </is>
       </c>
       <c r="E59" t="inlineStr">
         <is>
-          <t>Mixed feelings. The hardware is sturdy, but software integration is clunky and requires frequent resets. 3 out of 5 stars. Would definitely recommend checking it out!</t>
+          <t>Decent spot, nothing extraordinary. The food was okay, service was acceptable, and the prices were fair for the neighborhood. Hope this review helps someone make up their mind.</t>
         </is>
       </c>
       <c r="F59" t="n">
@@ -2534,11 +2534,11 @@
       </c>
       <c r="G59" t="inlineStr">
         <is>
-          <t>13.12.2024</t>
+          <t>01.02.2022</t>
         </is>
       </c>
       <c r="H59" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
     </row>
     <row r="60">
@@ -2547,34 +2547,34 @@
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t>REV-AMA-00500</t>
+          <t>REV-GOO-03195</t>
         </is>
       </c>
       <c r="C60" t="inlineStr">
         <is>
-          <t>Amazon</t>
+          <t>Google Locations</t>
         </is>
       </c>
       <c r="D60" t="inlineStr">
         <is>
-          <t>Anker 65W GaN Fast Charger</t>
+          <t>Metropolitan Dental Health Clinic</t>
         </is>
       </c>
       <c r="E60" t="inlineStr">
         <is>
-          <t>Average product. It gets the job done for everyday basic use, but nothing to write home about. Decent value for the budget price. #verifiedpurchase</t>
+          <t>Great atmosphere and delicious food! The pasta was freshly handmade and the wine selection was impressive. Service was attentive and friendly. Packaging was decent.</t>
         </is>
       </c>
       <c r="F60" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="G60" t="inlineStr">
         <is>
-          <t>05.09.2024</t>
+          <t>18.10.2022</t>
         </is>
       </c>
       <c r="H60" t="n">
-        <v>10</v>
+        <v>1</v>
       </c>
     </row>
     <row r="61">
@@ -2583,22 +2583,22 @@
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>REV-AMA-01991</t>
+          <t>REV-GOO-04235</t>
         </is>
       </c>
       <c r="C61" t="inlineStr">
         <is>
-          <t>Amazon</t>
+          <t>Google Locations</t>
         </is>
       </c>
       <c r="D61" t="inlineStr">
         <is>
-          <t>Anker 65W GaN Fast Charger</t>
+          <t>Metropolitan Dental Health Clinic</t>
         </is>
       </c>
       <c r="E61" t="inlineStr">
         <is>
-          <t>Review update after 3 months: Much better than my previous one. Sleek, fast, and intuitive. Dropped one star because the companion app occasionally desyncs.</t>
+          <t>Summary: Great atmosphere and delicious food! The pasta was freshly handmade and the wine selection was impressive. Service was attentive and friendly.</t>
         </is>
       </c>
       <c r="F61" t="n">
@@ -2606,11 +2606,11 @@
       </c>
       <c r="G61" t="inlineStr">
         <is>
-          <t>14.11.2023</t>
+          <t>07.08.2023</t>
         </is>
       </c>
       <c r="H61" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
     </row>
   </sheetData>

</xml_diff>